<commit_message>
RSVP stats: first record (pipeline integration test)
</commit_message>
<xml_diff>
--- a/嘉宾回执统计.xlsx
+++ b/嘉宾回执统计.xlsx
@@ -73,9 +73,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -446,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -477,21 +480,39 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>联调测试</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17 11:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>0 份回执</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>1 份回执</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Excel regenerated with dedup logic (integration test row, latest count)
</commit_message>
<xml_diff>
--- a/嘉宾回执统计.xlsx
+++ b/嘉宾回执统计.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="回执统计" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="回执统计" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,11 +490,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 11:02</t>
+          <t>2026-08-17 11:08</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
     </row>

</xml_diff>